<commit_message>
feat: publish menu composition and partner spotlight
</commit_message>
<xml_diff>
--- a/public/templates/delikreol_template_import_traiteurs.xlsx
+++ b/public/templates/delikreol_template_import_traiteurs.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" r:id="Red5a32022aa54c6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rd152559cbb074367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" r:id="R457a04cda62442a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R55fb55dffbaf4126"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -91,8 +91,18 @@
         <x:fgColor rgb="FFD1FAE5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7A321F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF7A321F"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -108,11 +118,25 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE8D8C4"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE8D8C4"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE8D8C4"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE8D8C4"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -174,6 +198,74 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -380,56 +472,100 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="4.21999979019165" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.110000133514404" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="4.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="10" t="str">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="53" t="str">
         <x:v>nom</x:v>
       </x:c>
-      <x:c r="B1" s="10" t="str">
+      <x:c r="B1" s="53" t="str">
         <x:v>prix</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="53" t="str">
         <x:v>description</x:v>
       </x:c>
-      <x:c r="D1" s="10" t="str">
+      <x:c r="D1" s="53" t="str">
         <x:v>categorie</x:v>
       </x:c>
-      <x:c r="E1" s="10" t="str">
+      <x:c r="E1" s="53" t="str">
         <x:v>stock</x:v>
       </x:c>
-      <x:c r="F1" s="10" t="str">
+      <x:c r="F1" s="53" t="str">
         <x:v>image_url</x:v>
       </x:c>
-      <x:c r="G1" s="10" t="str">
+      <x:c r="G1" s="53" t="str">
         <x:v>accompagnements</x:v>
       </x:c>
-      <x:c r="H1" s="10" t="str">
+      <x:c r="H1" s="53" t="str">
         <x:v>boissons</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="str">
+      <x:c r="I1" s="53" t="str">
+        <x:v>sauces</x:v>
+      </x:c>
+      <x:c r="J1" s="54" t="str">
+        <x:v>accompagnements_inclus</x:v>
+      </x:c>
+      <x:c r="K1" s="54" t="str">
+        <x:v>boissons_inclus</x:v>
+      </x:c>
+      <x:c r="L1" s="54" t="str">
+        <x:v>sauces_inclus</x:v>
+      </x:c>
+      <x:c r="M1" s="54" t="str">
         <x:v>traiteur</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="11"/>
-      <x:c r="B2" s="12"/>
-      <x:c r="C2" s="11"/>
-      <x:c r="D2" s="11"/>
-      <x:c r="E2" s="13"/>
-      <x:c r="F2" s="11"/>
-      <x:c r="G2" s="11"/>
-      <x:c r="H2" s="11"/>
-      <x:c r="I2" s="11"/>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="32" t="str">
+        <x:v>Colombo de poulet</x:v>
+      </x:c>
+      <x:c r="B2" s="33" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="C2" s="32" t="str">
+        <x:v>Poulet mijoté aux épices douces</x:v>
+      </x:c>
+      <x:c r="D2" s="32" t="str">
+        <x:v>Menu</x:v>
+      </x:c>
+      <x:c r="E2" s="34" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F2" s="32" t="str"/>
+      <x:c r="G2" s="32" t="str">
+        <x:v>Riz;Légumes pays</x:v>
+      </x:c>
+      <x:c r="H2" s="32" t="str">
+        <x:v>Jus local;Eau</x:v>
+      </x:c>
+      <x:c r="I2" s="32" t="str">
+        <x:v>Sauce chien;Sans sauce</x:v>
+      </x:c>
+      <x:c r="J2" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K2" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L2" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M2" s="41" t="str">
+        <x:v>Nom du traiteur</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11"/>
@@ -1543,10 +1679,10 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="73.77999877929688" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
   </x:cols>
@@ -1569,9 +1705,9 @@
       <x:c r="E2" s="24"/>
       <x:c r="F2" s="24"/>
     </x:row>
-    <x:row r="3" ht="28" customHeight="1">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="25" t="str">
-        <x:v>1. Remplissez uniquement la feuille « Import », une ligne par produit.</x:v>
+        <x:v>1. Remplissez la feuille « Import », une ligne par produit.</x:v>
       </x:c>
       <x:c r="B3" s="25"/>
       <x:c r="C3" s="25"/>
@@ -1579,9 +1715,9 @@
       <x:c r="E3" s="25"/>
       <x:c r="F3" s="25"/>
     </x:row>
-    <x:row r="4" ht="28" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="25" t="str">
-        <x:v>2. Les colonnes nom et prix sont obligatoires. Le stock vide sera mis à 15 par défaut.</x:v>
+        <x:v>2. Les colonnes nom et prix sont obligatoires. Le stock vide sera mis à 15.</x:v>
       </x:c>
       <x:c r="B4" s="25"/>
       <x:c r="C4" s="25"/>
@@ -1589,9 +1725,9 @@
       <x:c r="E4" s="25"/>
       <x:c r="F4" s="25"/>
     </x:row>
-    <x:row r="5" ht="28" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="25" t="str">
-        <x:v>3. Dans accompagnements et boissons, séparez plusieurs éléments avec un point-virgule ;</x:v>
+        <x:v>3. Séparez plusieurs accompagnements, boissons ou sauces avec un point-virgule.</x:v>
       </x:c>
       <x:c r="B5" s="25"/>
       <x:c r="C5" s="25"/>
@@ -1599,9 +1735,9 @@
       <x:c r="E5" s="25"/>
       <x:c r="F5" s="25"/>
     </x:row>
-    <x:row r="6" ht="28" customHeight="1">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="25" t="str">
-        <x:v>4. image_url doit être une URL publique directe vers la photo (ou laissez vide).</x:v>
+        <x:v>4. Pour un menu, indiquez le nombre de choix inclus dans les trois colonnes « inclus ».</x:v>
       </x:c>
       <x:c r="B6" s="25"/>
       <x:c r="C6" s="25"/>
@@ -1609,9 +1745,9 @@
       <x:c r="E6" s="25"/>
       <x:c r="F6" s="25"/>
     </x:row>
-    <x:row r="7" ht="28" customHeight="1">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="25" t="str">
-        <x:v>5. Avant l’envoi dans l’application : Fichier → Enregistrer sous → CSV UTF-8 (séparateur ; si proposé).</x:v>
+        <x:v>5. image_url accepte une URL publique. Vous pouvez aussi importer les photos en lot dans l’espace partenaire.</x:v>
       </x:c>
       <x:c r="B7" s="25"/>
       <x:c r="C7" s="25"/>
@@ -1619,9 +1755,9 @@
       <x:c r="E7" s="25"/>
       <x:c r="F7" s="25"/>
     </x:row>
-    <x:row r="8" ht="28" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="25" t="str">
-        <x:v>6. N’envoyez pas le fichier Excel .xlsx directement dans le bouton actuel : l’import publié attend un CSV.</x:v>
+        <x:v>6. Nommez chaque photo comme le produit, par exemple colombo-de-poulet.jpg.</x:v>
       </x:c>
       <x:c r="B8" s="25"/>
       <x:c r="C8" s="25"/>
@@ -1629,173 +1765,209 @@
       <x:c r="E8" s="25"/>
       <x:c r="F8" s="25"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="24"/>
-      <x:c r="B9" s="24"/>
-      <x:c r="C9" s="24"/>
-      <x:c r="D9" s="24"/>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="49" t="str">
+        <x:v>7. Enregistrez ensuite la feuille Import en CSV UTF-8 avant de l’importer.</x:v>
+      </x:c>
+      <x:c r="B9" s="49"/>
+      <x:c r="C9" s="49"/>
+      <x:c r="D9" s="49"/>
       <x:c r="E9" s="24"/>
       <x:c r="F9" s="24"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="26" t="str">
-        <x:v>Colonne</x:v>
-      </x:c>
-      <x:c r="B10" s="26" t="str">
-        <x:v>Obligatoire</x:v>
-      </x:c>
-      <x:c r="C10" s="26" t="str">
-        <x:v>Exemple</x:v>
-      </x:c>
-      <x:c r="D10" s="26" t="str">
-        <x:v>Règle</x:v>
-      </x:c>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="50"/>
+      <x:c r="B10" s="50"/>
+      <x:c r="C10" s="50"/>
+      <x:c r="D10" s="50"/>
       <x:c r="E10" s="27" t="str"/>
       <x:c r="F10" s="27" t="str"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="28" t="str">
-        <x:v>nom</x:v>
-      </x:c>
-      <x:c r="B11" s="28" t="str">
-        <x:v>Oui</x:v>
-      </x:c>
-      <x:c r="C11" s="28" t="str">
-        <x:v>Colombo de poulet</x:v>
-      </x:c>
-      <x:c r="D11" s="28" t="str">
-        <x:v>Nom visible du produit</x:v>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="55" t="str">
+        <x:v>Colonne</x:v>
+      </x:c>
+      <x:c r="B11" s="55" t="str">
+        <x:v>Obligatoire</x:v>
+      </x:c>
+      <x:c r="C11" s="55" t="str">
+        <x:v>Exemple</x:v>
+      </x:c>
+      <x:c r="D11" s="55" t="str">
+        <x:v>Règle</x:v>
       </x:c>
       <x:c r="E11" s="24"/>
       <x:c r="F11" s="24"/>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="28" t="str">
-        <x:v>prix</x:v>
-      </x:c>
-      <x:c r="B12" s="28" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="11" t="str">
+        <x:v>nom</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
         <x:v>Oui</x:v>
       </x:c>
-      <x:c r="C12" s="28" t="str">
-        <x:v>12.50</x:v>
-      </x:c>
-      <x:c r="D12" s="28" t="str">
-        <x:v>Prix en euros, sans symbole €</x:v>
+      <x:c r="C12" s="11" t="str">
+        <x:v>Colombo de poulet</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>Nom visible du produit</x:v>
       </x:c>
       <x:c r="E12" s="24"/>
       <x:c r="F12" s="24"/>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="28" t="str">
-        <x:v>description</x:v>
-      </x:c>
-      <x:c r="B13" s="28" t="str">
-        <x:v>Non</x:v>
-      </x:c>
-      <x:c r="C13" s="28" t="str">
-        <x:v>Poulet mijoté aux épices douces</x:v>
-      </x:c>
-      <x:c r="D13" s="28" t="str">
-        <x:v>Description courte</x:v>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="11" t="str">
+        <x:v>prix</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>Prix en euros</x:v>
       </x:c>
       <x:c r="E13" s="24"/>
       <x:c r="F13" s="24"/>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="28" t="str">
-        <x:v>categorie</x:v>
-      </x:c>
-      <x:c r="B14" s="28" t="str">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="11" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C14" s="28" t="str">
-        <x:v>Plat</x:v>
-      </x:c>
-      <x:c r="D14" s="28" t="str">
-        <x:v>Plat, Menu, Dessert, Boisson, Buffet, Brunch ou Autre</x:v>
+      <x:c r="C14" s="11" t="str">
+        <x:v>Poulet mijoté</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>Description courte</x:v>
       </x:c>
       <x:c r="E14" s="24"/>
       <x:c r="F14" s="24"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="28" t="str">
-        <x:v>stock</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="str">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="11" t="str">
+        <x:v>categorie</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C15" s="28" t="str">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D15" s="28" t="str">
-        <x:v>Nombre entier ; 15 par défaut si vide</x:v>
+      <x:c r="C15" s="11" t="str">
+        <x:v>Menu</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>Plat, Menu, Dessert, Boisson, Buffet, Brunch ou Autre</x:v>
       </x:c>
       <x:c r="E15" s="24"/>
       <x:c r="F15" s="24"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="28" t="str">
-        <x:v>image_url</x:v>
-      </x:c>
-      <x:c r="B16" s="28" t="str">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="11" t="str">
+        <x:v>stock</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C16" s="28" t="str">
-        <x:v>https://…/photo.jpg</x:v>
-      </x:c>
-      <x:c r="D16" s="28" t="str">
-        <x:v>URL publique de l’image</x:v>
+      <x:c r="C16" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
+        <x:v>15 par défaut si vide</x:v>
       </x:c>
       <x:c r="E16" s="24"/>
       <x:c r="F16" s="24"/>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="28" t="str">
-        <x:v>accompagnements</x:v>
-      </x:c>
-      <x:c r="B17" s="28" t="str">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="11" t="str">
+        <x:v>image_url</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C17" s="28" t="str">
-        <x:v>Riz;Salade</x:v>
-      </x:c>
-      <x:c r="D17" s="28" t="str">
-        <x:v>Plusieurs valeurs séparées par ;</x:v>
+      <x:c r="C17" s="11" t="str">
+        <x:v>https://…/photo.jpg</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
+        <x:v>URL publique ou import photo séparé</x:v>
       </x:c>
       <x:c r="E17" s="24"/>
       <x:c r="F17" s="24"/>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="28" t="str">
-        <x:v>boissons</x:v>
-      </x:c>
-      <x:c r="B18" s="28" t="str">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="11" t="str">
+        <x:v>accompagnements</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C18" s="28" t="str">
-        <x:v>Jus bissap;Eau</x:v>
-      </x:c>
-      <x:c r="D18" s="28" t="str">
-        <x:v>Plusieurs valeurs séparées par ;</x:v>
+      <x:c r="C18" s="11" t="str">
+        <x:v>Riz;Légumes pays</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
+        <x:v>Choix séparés par ;</x:v>
       </x:c>
       <x:c r="E18" s="24"/>
       <x:c r="F18" s="24"/>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="28" t="str">
-        <x:v>traiteur</x:v>
-      </x:c>
-      <x:c r="B19" s="28" t="str">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="11" t="str">
+        <x:v>boissons</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="str">
         <x:v>Non</x:v>
       </x:c>
-      <x:c r="C19" s="28" t="str">
-        <x:v>Nom du traiteur</x:v>
-      </x:c>
-      <x:c r="D19" s="28" t="str">
-        <x:v>Utilisé par l’administration ; ignoré par le traiteur</x:v>
+      <x:c r="C19" s="11" t="str">
+        <x:v>Jus local;Eau</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="str">
+        <x:v>Choix séparés par ;</x:v>
       </x:c>
       <x:c r="E19" s="24"/>
       <x:c r="F19" s="24"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="52" t="str">
+        <x:v>sauces</x:v>
+      </x:c>
+      <x:c r="B20" s="52" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="C20" s="52" t="str">
+        <x:v>Sauce chien;Sans sauce</x:v>
+      </x:c>
+      <x:c r="D20" s="52" t="str">
+        <x:v>Choix séparés par ;</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="52" t="str">
+        <x:v>accompagnements_inclus / boissons_inclus / sauces_inclus</x:v>
+      </x:c>
+      <x:c r="B21" s="52" t="str">
+        <x:v>Pour un menu</x:v>
+      </x:c>
+      <x:c r="C21" s="52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="52" t="str">
+        <x:v>Nombre exact de cases que le client doit cocher</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="52" t="str">
+        <x:v>traiteur</x:v>
+      </x:c>
+      <x:c r="B22" s="52" t="str">
+        <x:v>Admin seulement</x:v>
+      </x:c>
+      <x:c r="C22" s="52" t="str">
+        <x:v>Nom du traiteur</x:v>
+      </x:c>
+      <x:c r="D22" s="52" t="str">
+        <x:v>Ignoré dans l’espace traiteur</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>